<commit_message>
Mac dinh giao dien sang, lap day 4 tab phan loai con trong bang 8 tin that
- index.html: mac dinh theme sang cho nguoi xem lan dau (bo logic tu chon
  theo gio trong ngay), ai bam nut chuyen doi van duoc nho lua chon rieng.
- Them 8 hoat dong that (nguon hvcsnd.edu.vn) cho 4 danh muc dang trong:
  Chuyen doi so (2), Doi moi sang tao (2), Nghien cuu khoa hoc (2), Khac
  (3, hoan thien tu chinh cac dong link nguoi dung da dan san trong Excel
  nhung chua kip dien tieu de/ngay).
- Sua category 1 su kien tu "an-ninh-mang" sang "khac" cho khop voi ban
  cap nhat moi nhat cua nguoi dung trong uploads/mau-nhap-hoat-dong.xlsx.
</commit_message>
<xml_diff>
--- a/uploads/mau-nhap-hoat-dong.xlsx
+++ b/uploads/mau-nhap-hoat-dong.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/macbook/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\VUONGNQ\Desktop\TUYEN_TRUYEN\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FA7EC9D-12FD-3645-847D-534C74B83B46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{717425BC-9FC3-4944-A341-99C08D32AEA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nhap hoat dong" sheetId="1" r:id="rId1"/>
@@ -399,7 +399,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -440,11 +440,11 @@
     <xf numFmtId="14" fontId="9" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -751,20 +751,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" style="6" customWidth="1"/>
-    <col min="2" max="2" width="54.5" style="6" customWidth="1"/>
+    <col min="2" max="2" width="54.44140625" style="6" customWidth="1"/>
     <col min="3" max="3" width="18" style="6" customWidth="1"/>
-    <col min="4" max="4" width="27.83203125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="27.77734375" style="6" customWidth="1"/>
     <col min="5" max="5" width="16" style="6" customWidth="1"/>
-    <col min="6" max="6" width="34.5" style="6" customWidth="1"/>
+    <col min="6" max="6" width="34.44140625" style="6" customWidth="1"/>
     <col min="7" max="7" width="46" style="6" customWidth="1"/>
     <col min="8" max="10" width="30" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.83203125" style="6"/>
+    <col min="11" max="16384" width="8.77734375" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="34" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -796,7 +796,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="7">
         <v>1</v>
       </c>
@@ -826,7 +826,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="43.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -844,7 +844,7 @@
       <c r="I3" s="9"/>
       <c r="J3" s="9"/>
     </row>
-    <row r="4" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="43.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -862,7 +862,7 @@
       <c r="I4" s="9"/>
       <c r="J4" s="9"/>
     </row>
-    <row r="5" spans="1:10" ht="44" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="43.95" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>3</v>
       </c>
@@ -880,7 +880,7 @@
       <c r="I5" s="9"/>
       <c r="J5" s="9"/>
     </row>
-    <row r="6" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
         <v>12</v>
       </c>
@@ -902,7 +902,7 @@
       <c r="I6" s="9"/>
       <c r="J6" s="9"/>
     </row>
-    <row r="7" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
         <v>4</v>
       </c>
@@ -926,7 +926,7 @@
       <c r="I7" s="9"/>
       <c r="J7" s="9"/>
     </row>
-    <row r="8" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="8">
         <v>5</v>
       </c>
@@ -950,7 +950,7 @@
       <c r="I8" s="9"/>
       <c r="J8" s="9"/>
     </row>
-    <row r="9" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="8">
         <v>6</v>
       </c>
@@ -974,7 +974,7 @@
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
     </row>
-    <row r="10" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="8"/>
       <c r="B10" s="9" t="s">
         <v>58</v>
@@ -996,7 +996,7 @@
       <c r="I10" s="9"/>
       <c r="J10" s="9"/>
     </row>
-    <row r="11" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
         <v>7</v>
       </c>
@@ -1020,7 +1020,7 @@
       <c r="I11" s="9"/>
       <c r="J11" s="9"/>
     </row>
-    <row r="12" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="8">
         <v>8</v>
       </c>
@@ -1044,7 +1044,7 @@
       <c r="I12" s="9"/>
       <c r="J12" s="9"/>
     </row>
-    <row r="13" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
         <v>9</v>
       </c>
@@ -1068,7 +1068,7 @@
       <c r="I13" s="9"/>
       <c r="J13" s="9"/>
     </row>
-    <row r="14" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="8">
         <v>10</v>
       </c>
@@ -1092,7 +1092,7 @@
       <c r="I14" s="9"/>
       <c r="J14" s="9"/>
     </row>
-    <row r="15" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="8">
         <v>11</v>
       </c>
@@ -1100,7 +1100,7 @@
         <v>45</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="D15" s="4" t="s">
         <v>40</v>
@@ -1116,7 +1116,7 @@
       <c r="I15" s="9"/>
       <c r="J15" s="9"/>
     </row>
-    <row r="16" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="8">
         <v>12</v>
       </c>
@@ -1130,7 +1130,7 @@
       <c r="I16" s="9"/>
       <c r="J16" s="9"/>
     </row>
-    <row r="17" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
         <v>9</v>
       </c>
@@ -1144,7 +1144,7 @@
       <c r="I17" s="9"/>
       <c r="J17" s="9"/>
     </row>
-    <row r="18" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
         <v>10</v>
       </c>
@@ -1158,7 +1158,7 @@
       <c r="I18" s="9"/>
       <c r="J18" s="9"/>
     </row>
-    <row r="19" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="8">
         <v>11</v>
       </c>
@@ -1172,7 +1172,7 @@
       <c r="I19" s="9"/>
       <c r="J19" s="9"/>
     </row>
-    <row r="20" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <v>12</v>
       </c>
@@ -1186,7 +1186,7 @@
       <c r="I20" s="9"/>
       <c r="J20" s="9"/>
     </row>
-    <row r="21" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="8">
         <v>13</v>
       </c>
@@ -1200,7 +1200,7 @@
       <c r="I21" s="9"/>
       <c r="J21" s="9"/>
     </row>
-    <row r="22" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>14</v>
       </c>
@@ -1214,7 +1214,7 @@
       <c r="I22" s="9"/>
       <c r="J22" s="9"/>
     </row>
-    <row r="23" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>15</v>
       </c>
@@ -1228,7 +1228,7 @@
       <c r="I23" s="9"/>
       <c r="J23" s="9"/>
     </row>
-    <row r="24" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>16</v>
       </c>
@@ -1242,7 +1242,7 @@
       <c r="I24" s="9"/>
       <c r="J24" s="9"/>
     </row>
-    <row r="25" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>17</v>
       </c>
@@ -1256,7 +1256,7 @@
       <c r="I25" s="9"/>
       <c r="J25" s="9"/>
     </row>
-    <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
         <v>18</v>
       </c>
@@ -1270,7 +1270,7 @@
       <c r="I26" s="9"/>
       <c r="J26" s="9"/>
     </row>
-    <row r="27" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
         <v>19</v>
       </c>
@@ -1284,7 +1284,7 @@
       <c r="I27" s="9"/>
       <c r="J27" s="9"/>
     </row>
-    <row r="28" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>20</v>
       </c>
@@ -1298,7 +1298,7 @@
       <c r="I28" s="9"/>
       <c r="J28" s="9"/>
     </row>
-    <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="8">
         <v>21</v>
       </c>
@@ -1312,7 +1312,7 @@
       <c r="I29" s="9"/>
       <c r="J29" s="9"/>
     </row>
-    <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="8">
         <v>22</v>
       </c>
@@ -1326,7 +1326,7 @@
       <c r="I30" s="9"/>
       <c r="J30" s="9"/>
     </row>
-    <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="8">
         <v>23</v>
       </c>
@@ -1340,7 +1340,7 @@
       <c r="I31" s="9"/>
       <c r="J31" s="9"/>
     </row>
-    <row r="32" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="8">
         <v>24</v>
       </c>
@@ -1354,7 +1354,7 @@
       <c r="I32" s="9"/>
       <c r="J32" s="9"/>
     </row>
-    <row r="33" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="8">
         <v>25</v>
       </c>
@@ -1368,7 +1368,7 @@
       <c r="I33" s="9"/>
       <c r="J33" s="9"/>
     </row>
-    <row r="34" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="8">
         <v>26</v>
       </c>
@@ -1382,7 +1382,7 @@
       <c r="I34" s="9"/>
       <c r="J34" s="9"/>
     </row>
-    <row r="35" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="8">
         <v>27</v>
       </c>
@@ -1396,7 +1396,7 @@
       <c r="I35" s="9"/>
       <c r="J35" s="9"/>
     </row>
-    <row r="36" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A36" s="8">
         <v>28</v>
       </c>
@@ -1410,7 +1410,7 @@
       <c r="I36" s="9"/>
       <c r="J36" s="9"/>
     </row>
-    <row r="37" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="8">
         <v>29</v>
       </c>
@@ -1424,7 +1424,7 @@
       <c r="I37" s="9"/>
       <c r="J37" s="9"/>
     </row>
-    <row r="38" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" ht="18" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="8">
         <v>30</v>
       </c>
@@ -1456,67 +1456,67 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="100" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="19" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="30" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="30" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="45" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:1" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="45" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:1" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>28</v>
       </c>

</xml_diff>